<commit_message>
Swiss DCF Model 1.0.0: Texte der Beispieldatei fuer das Repository angepasst
</commit_message>
<xml_diff>
--- a/dcf/swiss-dcf-example-v1.0.0.xlsx
+++ b/dcf/swiss-dcf-example-v1.0.0.xlsx
@@ -136,7 +136,7 @@
     <comment ref="C17" authorId="0">
       <text>
         <r>
-          <t>Comparison values, as on the website. WACC (CAPM): cost of capital from the CAPM inputs with the current risk-free rate. Implied WACC: the WACC at which the value per share equals the current share price (sheet Reverse DCF). Set WACC source = CAPM on Inputs to value with the CAPM WACC.</t>
+          <t>Comparison values. WACC (CAPM): cost of capital from the CAPM inputs with the current risk-free rate. Implied WACC: the WACC at which the value per share equals the current share price (sheet Reverse DCF). Set WACC source = CAPM on Inputs to value with the CAPM WACC.</t>
         </r>
       </text>
     </comment>
@@ -598,7 +598,7 @@
     <t>File</t>
   </si>
   <si>
-    <t>Model with your inputs from noelwalpert.com</t>
+    <t>Example with neutral illustrative values</t>
   </si>
   <si>
     <t>Currency and units</t>
@@ -712,7 +712,7 @@
     <t>Method</t>
   </si>
   <si>
-    <t>https://noelwalpert.com/tools/dcf-rechner (section "Für Fachleute")</t>
+    <t>dcf/README.md in the repository. Online: noelwalpert.com/tools/dcf-rechner</t>
   </si>
   <si>
     <t>Repository</t>
@@ -2544,7 +2544,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="37" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="37" ht="26" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B37" s="7" t="s">
         <v>44</v>
       </c>

</xml_diff>